<commit_message>
Log MQTT data 2026-08-17 14:59 UTC
</commit_message>
<xml_diff>
--- a/logs/raiv_tracker_2026-08-17.xlsx
+++ b/logs/raiv_tracker_2026-08-17.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1692"/>
+  <dimension ref="A1:F1752"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40957,7 +40957,6 @@
           <t>6</t>
         </is>
       </c>
-      <c r="E1465" t="inlineStr"/>
       <c r="F1465" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g2</t>
@@ -40985,7 +40984,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1466" t="inlineStr"/>
       <c r="F1466" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g3</t>
@@ -41013,7 +41011,6 @@
           <t>7</t>
         </is>
       </c>
-      <c r="E1467" t="inlineStr"/>
       <c r="F1467" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g4</t>
@@ -41041,7 +41038,6 @@
           <t>11</t>
         </is>
       </c>
-      <c r="E1468" t="inlineStr"/>
       <c r="F1468" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g5</t>
@@ -41069,7 +41065,6 @@
           <t>2</t>
         </is>
       </c>
-      <c r="E1469" t="inlineStr"/>
       <c r="F1469" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g6</t>
@@ -41097,7 +41092,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1470" t="inlineStr"/>
       <c r="F1470" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g7</t>
@@ -41125,7 +41119,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1471" t="inlineStr"/>
       <c r="F1471" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g13</t>
@@ -41153,7 +41146,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1472" t="inlineStr"/>
       <c r="F1472" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g15</t>
@@ -41181,7 +41173,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1473" t="inlineStr"/>
       <c r="F1473" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g17</t>
@@ -41209,7 +41200,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1474" t="inlineStr"/>
       <c r="F1474" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g18</t>
@@ -41237,7 +41227,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1475" t="inlineStr"/>
       <c r="F1475" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g19</t>
@@ -41265,7 +41254,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1476" t="inlineStr"/>
       <c r="F1476" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g22</t>
@@ -41293,7 +41281,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1477" t="inlineStr"/>
       <c r="F1477" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g23</t>
@@ -41321,7 +41308,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1478" t="inlineStr"/>
       <c r="F1478" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g24</t>
@@ -41349,7 +41335,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1479" t="inlineStr"/>
       <c r="F1479" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g25</t>
@@ -41377,7 +41362,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1480" t="inlineStr"/>
       <c r="F1480" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g33</t>
@@ -41405,7 +41389,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1481" t="inlineStr"/>
       <c r="F1481" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g34</t>
@@ -41433,7 +41416,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1482" t="inlineStr"/>
       <c r="F1482" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g36</t>
@@ -41461,7 +41443,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1483" t="inlineStr"/>
       <c r="F1483" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g40</t>
@@ -41489,7 +41470,6 @@
           <t>13</t>
         </is>
       </c>
-      <c r="E1484" t="inlineStr"/>
       <c r="F1484" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g1</t>
@@ -41517,7 +41497,6 @@
           <t>1166</t>
         </is>
       </c>
-      <c r="E1485" t="inlineStr"/>
       <c r="F1485" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g8</t>
@@ -41545,7 +41524,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1486" t="inlineStr"/>
       <c r="F1486" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g9</t>
@@ -41573,7 +41551,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E1487" t="inlineStr"/>
       <c r="F1487" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g10</t>
@@ -41601,7 +41578,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E1488" t="inlineStr"/>
       <c r="F1488" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g11</t>
@@ -41629,7 +41605,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E1489" t="inlineStr"/>
       <c r="F1489" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g12</t>
@@ -41657,7 +41632,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1490" t="inlineStr"/>
       <c r="F1490" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g14</t>
@@ -41685,7 +41659,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1491" t="inlineStr"/>
       <c r="F1491" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g16</t>
@@ -41713,7 +41686,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1492" t="inlineStr"/>
       <c r="F1492" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g20</t>
@@ -41741,7 +41713,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1493" t="inlineStr"/>
       <c r="F1493" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g21</t>
@@ -41769,7 +41740,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1494" t="inlineStr"/>
       <c r="F1494" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g26</t>
@@ -41797,7 +41767,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1495" t="inlineStr"/>
       <c r="F1495" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g27</t>
@@ -41825,7 +41794,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1496" t="inlineStr"/>
       <c r="F1496" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g28</t>
@@ -41853,7 +41821,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1497" t="inlineStr"/>
       <c r="F1497" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g29</t>
@@ -41881,7 +41848,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1498" t="inlineStr"/>
       <c r="F1498" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g30</t>
@@ -41909,7 +41875,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1499" t="inlineStr"/>
       <c r="F1499" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g31</t>
@@ -41937,7 +41902,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1500" t="inlineStr"/>
       <c r="F1500" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g32</t>
@@ -41965,7 +41929,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1501" t="inlineStr"/>
       <c r="F1501" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g35</t>
@@ -41993,7 +41956,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1502" t="inlineStr"/>
       <c r="F1502" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g37</t>
@@ -42021,7 +41983,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1503" t="inlineStr"/>
       <c r="F1503" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g38</t>
@@ -42049,7 +42010,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1504" t="inlineStr"/>
       <c r="F1504" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g39</t>
@@ -43001,7 +42961,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1538" t="inlineStr"/>
       <c r="F1538" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g2</t>
@@ -43029,7 +42988,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1539" t="inlineStr"/>
       <c r="F1539" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g3</t>
@@ -43057,7 +43015,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1540" t="inlineStr"/>
       <c r="F1540" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g1</t>
@@ -43085,7 +43042,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1541" t="inlineStr"/>
       <c r="F1541" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g4</t>
@@ -43113,7 +43069,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1542" t="inlineStr"/>
       <c r="F1542" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g5</t>
@@ -43141,7 +43096,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1543" t="inlineStr"/>
       <c r="F1543" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g7</t>
@@ -43169,7 +43123,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1544" t="inlineStr"/>
       <c r="F1544" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g6</t>
@@ -43197,7 +43150,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1545" t="inlineStr"/>
       <c r="F1545" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g10</t>
@@ -43225,7 +43177,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1546" t="inlineStr"/>
       <c r="F1546" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g8</t>
@@ -43253,7 +43204,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1547" t="inlineStr"/>
       <c r="F1547" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g9</t>
@@ -43281,7 +43231,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1548" t="inlineStr"/>
       <c r="F1548" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g11</t>
@@ -43309,7 +43258,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E1549" t="inlineStr"/>
       <c r="F1549" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g12</t>
@@ -43337,7 +43285,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1550" t="inlineStr"/>
       <c r="F1550" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g13</t>
@@ -43365,7 +43312,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1551" t="inlineStr"/>
       <c r="F1551" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g14</t>
@@ -43393,7 +43339,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1552" t="inlineStr"/>
       <c r="F1552" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g15</t>
@@ -43421,7 +43366,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1553" t="inlineStr"/>
       <c r="F1553" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g16</t>
@@ -43449,7 +43393,6 @@
           <t>22</t>
         </is>
       </c>
-      <c r="E1554" t="inlineStr"/>
       <c r="F1554" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g22</t>
@@ -43477,7 +43420,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1555" t="inlineStr"/>
       <c r="F1555" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g23</t>
@@ -43505,7 +43447,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1556" t="inlineStr"/>
       <c r="F1556" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g17</t>
@@ -43533,7 +43474,6 @@
           <t>1378</t>
         </is>
       </c>
-      <c r="E1557" t="inlineStr"/>
       <c r="F1557" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g18</t>
@@ -43561,7 +43501,6 @@
           <t>1347</t>
         </is>
       </c>
-      <c r="E1558" t="inlineStr"/>
       <c r="F1558" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g19</t>
@@ -43589,7 +43528,6 @@
           <t>6</t>
         </is>
       </c>
-      <c r="E1559" t="inlineStr"/>
       <c r="F1559" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g21</t>
@@ -43617,7 +43555,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1560" t="inlineStr"/>
       <c r="F1560" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g24</t>
@@ -43645,7 +43582,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1561" t="inlineStr"/>
       <c r="F1561" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g25</t>
@@ -43673,7 +43609,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1562" t="inlineStr"/>
       <c r="F1562" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g26</t>
@@ -43701,7 +43636,6 @@
           <t>147</t>
         </is>
       </c>
-      <c r="E1563" t="inlineStr"/>
       <c r="F1563" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g27</t>
@@ -43729,7 +43663,6 @@
           <t>46</t>
         </is>
       </c>
-      <c r="E1564" t="inlineStr"/>
       <c r="F1564" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g31</t>
@@ -43757,7 +43690,6 @@
           <t>30</t>
         </is>
       </c>
-      <c r="E1565" t="inlineStr"/>
       <c r="F1565" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g32</t>
@@ -43785,7 +43717,6 @@
           <t>41</t>
         </is>
       </c>
-      <c r="E1566" t="inlineStr"/>
       <c r="F1566" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g28</t>
@@ -43813,7 +43744,6 @@
           <t>43</t>
         </is>
       </c>
-      <c r="E1567" t="inlineStr"/>
       <c r="F1567" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g29</t>
@@ -43841,7 +43771,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1568" t="inlineStr"/>
       <c r="F1568" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g30</t>
@@ -43869,7 +43798,6 @@
           <t>30</t>
         </is>
       </c>
-      <c r="E1569" t="inlineStr"/>
       <c r="F1569" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g33</t>
@@ -43897,7 +43825,6 @@
           <t>31</t>
         </is>
       </c>
-      <c r="E1570" t="inlineStr"/>
       <c r="F1570" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g37</t>
@@ -43925,7 +43852,6 @@
           <t>30</t>
         </is>
       </c>
-      <c r="E1571" t="inlineStr"/>
       <c r="F1571" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g34</t>
@@ -43953,7 +43879,6 @@
           <t>31</t>
         </is>
       </c>
-      <c r="E1572" t="inlineStr"/>
       <c r="F1572" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g35</t>
@@ -43981,7 +43906,6 @@
           <t>30</t>
         </is>
       </c>
-      <c r="E1573" t="inlineStr"/>
       <c r="F1573" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g36</t>
@@ -44009,7 +43933,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1574" t="inlineStr"/>
       <c r="F1574" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g39</t>
@@ -44037,7 +43960,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1575" t="inlineStr"/>
       <c r="F1575" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g40</t>
@@ -44065,7 +43987,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1576" t="inlineStr"/>
       <c r="F1576" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g38</t>
@@ -46305,7 +46226,6 @@
           <t>1167</t>
         </is>
       </c>
-      <c r="E1656" t="inlineStr"/>
       <c r="F1656" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g8</t>
@@ -47315,6 +47235,1686 @@
         <v>11</v>
       </c>
       <c r="F1692" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1693">
+      <c r="A1693" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1693" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1693" t="inlineStr">
+        <is>
+          <t>CountLaidButton</t>
+        </is>
+      </c>
+      <c r="D1693" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E1693" t="inlineStr"/>
+      <c r="F1693" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1694">
+      <c r="A1694" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1694" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1694" t="inlineStr">
+        <is>
+          <t>CountLaidDetector</t>
+        </is>
+      </c>
+      <c r="D1694" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1694" t="inlineStr"/>
+      <c r="F1694" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g3</t>
+        </is>
+      </c>
+    </row>
+    <row r="1695">
+      <c r="A1695" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1695" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1695" t="inlineStr">
+        <is>
+          <t>CountLaidEncoder</t>
+        </is>
+      </c>
+      <c r="D1695" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E1695" t="inlineStr"/>
+      <c r="F1695" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g4</t>
+        </is>
+      </c>
+    </row>
+    <row r="1696">
+      <c r="A1696" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1696" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1696" t="inlineStr">
+        <is>
+          <t>CountLaid14in</t>
+        </is>
+      </c>
+      <c r="D1696" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E1696" t="inlineStr"/>
+      <c r="F1696" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g5</t>
+        </is>
+      </c>
+    </row>
+    <row r="1697">
+      <c r="A1697" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1697" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1697" t="inlineStr">
+        <is>
+          <t>CountLaid18in</t>
+        </is>
+      </c>
+      <c r="D1697" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E1697" t="inlineStr"/>
+      <c r="F1697" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1698">
+      <c r="A1698" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1698" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1698" t="inlineStr">
+        <is>
+          <t>CountLaidPandral</t>
+        </is>
+      </c>
+      <c r="D1698" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1698" t="inlineStr"/>
+      <c r="F1698" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g7</t>
+        </is>
+      </c>
+    </row>
+    <row r="1699">
+      <c r="A1699" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1699" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1699" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D1699" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E1699" t="inlineStr"/>
+      <c r="F1699" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1700">
+      <c r="A1700" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1700" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1700" t="inlineStr">
+        <is>
+          <t>usr_TPStime Hours10th</t>
+        </is>
+      </c>
+      <c r="D1700" t="inlineStr">
+        <is>
+          <t>1177</t>
+        </is>
+      </c>
+      <c r="E1700" t="inlineStr"/>
+      <c r="F1700" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g8</t>
+        </is>
+      </c>
+    </row>
+    <row r="1701">
+      <c r="A1701" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1701" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1701" t="inlineStr">
+        <is>
+          <t>usrTPS_miles xxx</t>
+        </is>
+      </c>
+      <c r="D1701" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1701" t="inlineStr"/>
+      <c r="F1701" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g9</t>
+        </is>
+      </c>
+    </row>
+    <row r="1702">
+      <c r="A1702" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1702" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1702" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D1702" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E1702" t="inlineStr"/>
+      <c r="F1702" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g10</t>
+        </is>
+      </c>
+    </row>
+    <row r="1703">
+      <c r="A1703" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1703" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1703" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D1703" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E1703" t="inlineStr"/>
+      <c r="F1703" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g11</t>
+        </is>
+      </c>
+    </row>
+    <row r="1704">
+      <c r="A1704" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1704" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1704" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D1704" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E1704" t="inlineStr"/>
+      <c r="F1704" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g12</t>
+        </is>
+      </c>
+    </row>
+    <row r="1705">
+      <c r="A1705" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1705" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1705" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D1705" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1705" t="inlineStr"/>
+      <c r="F1705" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g13</t>
+        </is>
+      </c>
+    </row>
+    <row r="1706">
+      <c r="A1706" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1706" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1706" t="inlineStr">
+        <is>
+          <t>CountAcceptedTotal</t>
+        </is>
+      </c>
+      <c r="D1706" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1706" t="inlineStr"/>
+      <c r="F1706" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g15</t>
+        </is>
+      </c>
+    </row>
+    <row r="1707">
+      <c r="A1707" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1707" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1707" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D1707" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1707" t="inlineStr"/>
+      <c r="F1707" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g17</t>
+        </is>
+      </c>
+    </row>
+    <row r="1708">
+      <c r="A1708" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1708" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1708" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D1708" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1708" t="inlineStr"/>
+      <c r="F1708" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g14</t>
+        </is>
+      </c>
+    </row>
+    <row r="1709">
+      <c r="A1709" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1709" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1709" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D1709" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1709" t="inlineStr"/>
+      <c r="F1709" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g18</t>
+        </is>
+      </c>
+    </row>
+    <row r="1710">
+      <c r="A1710" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1710" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1710" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D1710" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1710" t="inlineStr"/>
+      <c r="F1710" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g19</t>
+        </is>
+      </c>
+    </row>
+    <row r="1711">
+      <c r="A1711" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1711" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1711" t="inlineStr">
+        <is>
+          <t>day_Servotime Hours10th</t>
+        </is>
+      </c>
+      <c r="D1711" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1711" t="inlineStr"/>
+      <c r="F1711" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g22</t>
+        </is>
+      </c>
+    </row>
+    <row r="1712">
+      <c r="A1712" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1712" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1712" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D1712" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1712" t="inlineStr"/>
+      <c r="F1712" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g23</t>
+        </is>
+      </c>
+    </row>
+    <row r="1713">
+      <c r="A1713" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1713" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1713" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D1713" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1713" t="inlineStr"/>
+      <c r="F1713" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g24</t>
+        </is>
+      </c>
+    </row>
+    <row r="1714">
+      <c r="A1714" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1714" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1714" t="inlineStr">
+        <is>
+          <t>tk_ClearPos</t>
+        </is>
+      </c>
+      <c r="D1714" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1714" t="inlineStr"/>
+      <c r="F1714" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g25</t>
+        </is>
+      </c>
+    </row>
+    <row r="1715">
+      <c r="A1715" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1715" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1715" t="inlineStr">
+        <is>
+          <t>CountRejectedTotal</t>
+        </is>
+      </c>
+      <c r="D1715" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1715" t="inlineStr"/>
+      <c r="F1715" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g16</t>
+        </is>
+      </c>
+    </row>
+    <row r="1716">
+      <c r="A1716" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1716" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1716" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D1716" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1716" t="inlineStr"/>
+      <c r="F1716" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g20</t>
+        </is>
+      </c>
+    </row>
+    <row r="1717">
+      <c r="A1717" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1717" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1717" t="inlineStr">
+        <is>
+          <t>tk_Cycle hrs</t>
+        </is>
+      </c>
+      <c r="D1717" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1717" t="inlineStr"/>
+      <c r="F1717" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g21</t>
+        </is>
+      </c>
+    </row>
+    <row r="1718">
+      <c r="A1718" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1718" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1718" t="inlineStr">
+        <is>
+          <t>tk_Warmup</t>
+        </is>
+      </c>
+      <c r="D1718" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1718" t="inlineStr"/>
+      <c r="F1718" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g26</t>
+        </is>
+      </c>
+    </row>
+    <row r="1719">
+      <c r="A1719" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1719" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1719" t="inlineStr">
+        <is>
+          <t>FindingParts min</t>
+        </is>
+      </c>
+      <c r="D1719" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1719" t="inlineStr"/>
+      <c r="F1719" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g27</t>
+        </is>
+      </c>
+    </row>
+    <row r="1720">
+      <c r="A1720" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1720" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1720" t="inlineStr">
+        <is>
+          <t>PickingParts min</t>
+        </is>
+      </c>
+      <c r="D1720" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1720" t="inlineStr"/>
+      <c r="F1720" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g28</t>
+        </is>
+      </c>
+    </row>
+    <row r="1721">
+      <c r="A1721" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1721" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1721" t="inlineStr">
+        <is>
+          <t>PlacingParts min</t>
+        </is>
+      </c>
+      <c r="D1721" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1721" t="inlineStr"/>
+      <c r="F1721" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g29</t>
+        </is>
+      </c>
+    </row>
+    <row r="1722">
+      <c r="A1722" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1722" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1722" t="inlineStr">
+        <is>
+          <t>CountPickedReject14in</t>
+        </is>
+      </c>
+      <c r="D1722" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1722" t="inlineStr"/>
+      <c r="F1722" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1723">
+      <c r="A1723" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1723" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1723" t="inlineStr">
+        <is>
+          <t>temp_dsi</t>
+        </is>
+      </c>
+      <c r="D1723" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1723" t="inlineStr"/>
+      <c r="F1723" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g31</t>
+        </is>
+      </c>
+    </row>
+    <row r="1724">
+      <c r="A1724" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1724" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1724" t="inlineStr">
+        <is>
+          <t>temp_J2motor</t>
+        </is>
+      </c>
+      <c r="D1724" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1724" t="inlineStr"/>
+      <c r="F1724" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g33</t>
+        </is>
+      </c>
+    </row>
+    <row r="1725">
+      <c r="A1725" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1725" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1725" t="inlineStr">
+        <is>
+          <t>temp_J3motor</t>
+        </is>
+      </c>
+      <c r="D1725" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1725" t="inlineStr"/>
+      <c r="F1725" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g34</t>
+        </is>
+      </c>
+    </row>
+    <row r="1726">
+      <c r="A1726" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1726" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1726" t="inlineStr">
+        <is>
+          <t>temp_J5motor</t>
+        </is>
+      </c>
+      <c r="D1726" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1726" t="inlineStr"/>
+      <c r="F1726" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g36</t>
+        </is>
+      </c>
+    </row>
+    <row r="1727">
+      <c r="A1727" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1727" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1727" t="inlineStr">
+        <is>
+          <t>CountPickedReject18in</t>
+        </is>
+      </c>
+      <c r="D1727" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1727" t="inlineStr"/>
+      <c r="F1727" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1728">
+      <c r="A1728" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1728" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1728" t="inlineStr">
+        <is>
+          <t>temp_J1motor</t>
+        </is>
+      </c>
+      <c r="D1728" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1728" t="inlineStr"/>
+      <c r="F1728" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g32</t>
+        </is>
+      </c>
+    </row>
+    <row r="1729">
+      <c r="A1729" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1729" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1729" t="inlineStr">
+        <is>
+          <t>temp_J4motor</t>
+        </is>
+      </c>
+      <c r="D1729" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1729" t="inlineStr"/>
+      <c r="F1729" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g35</t>
+        </is>
+      </c>
+    </row>
+    <row r="1730">
+      <c r="A1730" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1730" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1730" t="inlineStr">
+        <is>
+          <t>temp_J6motor</t>
+        </is>
+      </c>
+      <c r="D1730" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1730" t="inlineStr"/>
+      <c r="F1730" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g37</t>
+        </is>
+      </c>
+    </row>
+    <row r="1731">
+      <c r="A1731" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1731" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1731" t="inlineStr">
+        <is>
+          <t>CountPickedRejectOTM</t>
+        </is>
+      </c>
+      <c r="D1731" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1731" t="inlineStr"/>
+      <c r="F1731" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g38</t>
+        </is>
+      </c>
+    </row>
+    <row r="1732">
+      <c r="A1732" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:58:13</t>
+        </is>
+      </c>
+      <c r="B1732" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1732" t="inlineStr">
+        <is>
+          <t>CountPickedRejectPandral</t>
+        </is>
+      </c>
+      <c r="D1732" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1732" t="inlineStr"/>
+      <c r="F1732" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g39</t>
+        </is>
+      </c>
+    </row>
+    <row r="1733">
+      <c r="A1733" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:59:00</t>
+        </is>
+      </c>
+      <c r="B1733" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1733" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D1733" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1733" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1733" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1734">
+      <c r="A1734" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:59:00</t>
+        </is>
+      </c>
+      <c r="B1734" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1734" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D1734" t="b">
+        <v>1</v>
+      </c>
+      <c r="E1734" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1734" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1735">
+      <c r="A1735" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:59:00</t>
+        </is>
+      </c>
+      <c r="B1735" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1735" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D1735" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1735" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1735" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1736">
+      <c r="A1736" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:59:00</t>
+        </is>
+      </c>
+      <c r="B1736" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1736" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D1736" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1736" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1736" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1737">
+      <c r="A1737" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:59:00</t>
+        </is>
+      </c>
+      <c r="B1737" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1737" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D1737" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1737" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1737" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1738">
+      <c r="A1738" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:59:00</t>
+        </is>
+      </c>
+      <c r="B1738" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1738" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D1738" t="n">
+        <v>7925</v>
+      </c>
+      <c r="E1738" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1738" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1739">
+      <c r="A1739" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:59:00</t>
+        </is>
+      </c>
+      <c r="B1739" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1739" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D1739" t="n">
+        <v>2770</v>
+      </c>
+      <c r="E1739" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1739" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1740">
+      <c r="A1740" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:59:00</t>
+        </is>
+      </c>
+      <c r="B1740" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1740" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D1740" t="n">
+        <v>5155</v>
+      </c>
+      <c r="E1740" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1740" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1741">
+      <c r="A1741" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:59:00</t>
+        </is>
+      </c>
+      <c r="B1741" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1741" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D1741" t="n">
+        <v>0.6504731774330139</v>
+      </c>
+      <c r="E1741" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1741" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1742">
+      <c r="A1742" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:59:00</t>
+        </is>
+      </c>
+      <c r="B1742" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1742" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D1742" t="n">
+        <v>0.3495268225669861</v>
+      </c>
+      <c r="E1742" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1742" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1743">
+      <c r="A1743" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:59:00</t>
+        </is>
+      </c>
+      <c r="B1743" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1743" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D1743" t="n">
+        <v>1378</v>
+      </c>
+      <c r="E1743" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1743" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1744">
+      <c r="A1744" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:59:00</t>
+        </is>
+      </c>
+      <c r="B1744" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1744" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D1744" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1744" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1744" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1745">
+      <c r="A1745" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:59:00</t>
+        </is>
+      </c>
+      <c r="B1745" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1745" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D1745" t="n">
+        <v>1347</v>
+      </c>
+      <c r="E1745" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1745" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1746">
+      <c r="A1746" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:59:00</t>
+        </is>
+      </c>
+      <c r="B1746" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1746" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D1746" t="n">
+        <v>0.9775036573410034</v>
+      </c>
+      <c r="E1746" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1746" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1747">
+      <c r="A1747" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:59:00</t>
+        </is>
+      </c>
+      <c r="B1747" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1747" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D1747" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1747" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1747" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1748">
+      <c r="A1748" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:59:00</t>
+        </is>
+      </c>
+      <c r="B1748" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1748" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D1748" t="n">
+        <v>10.43280792236328</v>
+      </c>
+      <c r="E1748" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1748" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1749">
+      <c r="A1749" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:59:00</t>
+        </is>
+      </c>
+      <c r="B1749" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1749" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D1749" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1749" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1749" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1750">
+      <c r="A1750" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:59:00</t>
+        </is>
+      </c>
+      <c r="B1750" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1750" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D1750" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1750" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1750" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1751">
+      <c r="A1751" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:59:00</t>
+        </is>
+      </c>
+      <c r="B1751" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1751" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D1751" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1751" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1751" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1752">
+      <c r="A1752" t="inlineStr">
+        <is>
+          <t>2026-08-17T14:59:00</t>
+        </is>
+      </c>
+      <c r="B1752" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1752" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D1752" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1752" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1752" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/plc</t>
         </is>

</xml_diff>

<commit_message>
Log MQTT data 2026-08-17 15:55 UTC
</commit_message>
<xml_diff>
--- a/logs/raiv_tracker_2026-08-17.xlsx
+++ b/logs/raiv_tracker_2026-08-17.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1752"/>
+  <dimension ref="A1:F1813"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -47261,7 +47261,6 @@
           <t>6</t>
         </is>
       </c>
-      <c r="E1693" t="inlineStr"/>
       <c r="F1693" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g2</t>
@@ -47289,7 +47288,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1694" t="inlineStr"/>
       <c r="F1694" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g3</t>
@@ -47317,7 +47315,6 @@
           <t>7</t>
         </is>
       </c>
-      <c r="E1695" t="inlineStr"/>
       <c r="F1695" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g4</t>
@@ -47345,7 +47342,6 @@
           <t>11</t>
         </is>
       </c>
-      <c r="E1696" t="inlineStr"/>
       <c r="F1696" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g5</t>
@@ -47373,7 +47369,6 @@
           <t>2</t>
         </is>
       </c>
-      <c r="E1697" t="inlineStr"/>
       <c r="F1697" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g6</t>
@@ -47401,7 +47396,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1698" t="inlineStr"/>
       <c r="F1698" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g7</t>
@@ -47429,7 +47423,6 @@
           <t>13</t>
         </is>
       </c>
-      <c r="E1699" t="inlineStr"/>
       <c r="F1699" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g1</t>
@@ -47457,7 +47450,6 @@
           <t>1177</t>
         </is>
       </c>
-      <c r="E1700" t="inlineStr"/>
       <c r="F1700" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g8</t>
@@ -47485,7 +47477,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1701" t="inlineStr"/>
       <c r="F1701" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g9</t>
@@ -47513,7 +47504,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E1702" t="inlineStr"/>
       <c r="F1702" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g10</t>
@@ -47541,7 +47531,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E1703" t="inlineStr"/>
       <c r="F1703" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g11</t>
@@ -47569,7 +47558,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E1704" t="inlineStr"/>
       <c r="F1704" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g12</t>
@@ -47597,7 +47585,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1705" t="inlineStr"/>
       <c r="F1705" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g13</t>
@@ -47625,7 +47612,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1706" t="inlineStr"/>
       <c r="F1706" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g15</t>
@@ -47653,7 +47639,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1707" t="inlineStr"/>
       <c r="F1707" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g17</t>
@@ -47681,7 +47666,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1708" t="inlineStr"/>
       <c r="F1708" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g14</t>
@@ -47709,7 +47693,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1709" t="inlineStr"/>
       <c r="F1709" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g18</t>
@@ -47737,7 +47720,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1710" t="inlineStr"/>
       <c r="F1710" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g19</t>
@@ -47765,7 +47747,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1711" t="inlineStr"/>
       <c r="F1711" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g22</t>
@@ -47793,7 +47774,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1712" t="inlineStr"/>
       <c r="F1712" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g23</t>
@@ -47821,7 +47801,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1713" t="inlineStr"/>
       <c r="F1713" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g24</t>
@@ -47849,7 +47828,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1714" t="inlineStr"/>
       <c r="F1714" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g25</t>
@@ -47877,7 +47855,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1715" t="inlineStr"/>
       <c r="F1715" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g16</t>
@@ -47905,7 +47882,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1716" t="inlineStr"/>
       <c r="F1716" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g20</t>
@@ -47933,7 +47909,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1717" t="inlineStr"/>
       <c r="F1717" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g21</t>
@@ -47961,7 +47936,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1718" t="inlineStr"/>
       <c r="F1718" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g26</t>
@@ -47989,7 +47963,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1719" t="inlineStr"/>
       <c r="F1719" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g27</t>
@@ -48017,7 +47990,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1720" t="inlineStr"/>
       <c r="F1720" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g28</t>
@@ -48045,7 +48017,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1721" t="inlineStr"/>
       <c r="F1721" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g29</t>
@@ -48073,7 +48044,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1722" t="inlineStr"/>
       <c r="F1722" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g30</t>
@@ -48101,7 +48071,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1723" t="inlineStr"/>
       <c r="F1723" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g31</t>
@@ -48129,7 +48098,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1724" t="inlineStr"/>
       <c r="F1724" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g33</t>
@@ -48157,7 +48125,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1725" t="inlineStr"/>
       <c r="F1725" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g34</t>
@@ -48185,7 +48152,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1726" t="inlineStr"/>
       <c r="F1726" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g36</t>
@@ -48213,7 +48179,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1727" t="inlineStr"/>
       <c r="F1727" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g40</t>
@@ -48241,7 +48206,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1728" t="inlineStr"/>
       <c r="F1728" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g32</t>
@@ -48269,7 +48233,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1729" t="inlineStr"/>
       <c r="F1729" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g35</t>
@@ -48297,7 +48260,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1730" t="inlineStr"/>
       <c r="F1730" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g37</t>
@@ -48325,7 +48287,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1731" t="inlineStr"/>
       <c r="F1731" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g38</t>
@@ -48353,7 +48314,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1732" t="inlineStr"/>
       <c r="F1732" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g39</t>
@@ -48915,6 +48875,1714 @@
         <v>3</v>
       </c>
       <c r="F1752" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1753">
+      <c r="A1753" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1753" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1753" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D1753" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E1753" t="inlineStr"/>
+      <c r="F1753" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1754">
+      <c r="A1754" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1754" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1754" t="inlineStr">
+        <is>
+          <t>usr_TPStime Hours10th</t>
+        </is>
+      </c>
+      <c r="D1754" t="inlineStr">
+        <is>
+          <t>1186</t>
+        </is>
+      </c>
+      <c r="E1754" t="inlineStr"/>
+      <c r="F1754" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g8</t>
+        </is>
+      </c>
+    </row>
+    <row r="1755">
+      <c r="A1755" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1755" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1755" t="inlineStr">
+        <is>
+          <t>usrTPS_miles xxx</t>
+        </is>
+      </c>
+      <c r="D1755" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1755" t="inlineStr"/>
+      <c r="F1755" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g9</t>
+        </is>
+      </c>
+    </row>
+    <row r="1756">
+      <c r="A1756" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1756" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1756" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D1756" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E1756" t="inlineStr"/>
+      <c r="F1756" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g10</t>
+        </is>
+      </c>
+    </row>
+    <row r="1757">
+      <c r="A1757" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1757" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1757" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D1757" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E1757" t="inlineStr"/>
+      <c r="F1757" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g11</t>
+        </is>
+      </c>
+    </row>
+    <row r="1758">
+      <c r="A1758" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1758" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1758" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D1758" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E1758" t="inlineStr"/>
+      <c r="F1758" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g12</t>
+        </is>
+      </c>
+    </row>
+    <row r="1759">
+      <c r="A1759" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1759" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1759" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D1759" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1759" t="inlineStr"/>
+      <c r="F1759" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g14</t>
+        </is>
+      </c>
+    </row>
+    <row r="1760">
+      <c r="A1760" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1760" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1760" t="inlineStr">
+        <is>
+          <t>CountRejectedTotal</t>
+        </is>
+      </c>
+      <c r="D1760" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1760" t="inlineStr"/>
+      <c r="F1760" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g16</t>
+        </is>
+      </c>
+    </row>
+    <row r="1761">
+      <c r="A1761" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1761" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1761" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D1761" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1761" t="inlineStr"/>
+      <c r="F1761" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g20</t>
+        </is>
+      </c>
+    </row>
+    <row r="1762">
+      <c r="A1762" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1762" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1762" t="inlineStr">
+        <is>
+          <t>tk_Cycle hrs</t>
+        </is>
+      </c>
+      <c r="D1762" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1762" t="inlineStr"/>
+      <c r="F1762" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g21</t>
+        </is>
+      </c>
+    </row>
+    <row r="1763">
+      <c r="A1763" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1763" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1763" t="inlineStr">
+        <is>
+          <t>tk_Warmup</t>
+        </is>
+      </c>
+      <c r="D1763" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1763" t="inlineStr"/>
+      <c r="F1763" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g26</t>
+        </is>
+      </c>
+    </row>
+    <row r="1764">
+      <c r="A1764" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1764" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1764" t="inlineStr">
+        <is>
+          <t>FindingParts min</t>
+        </is>
+      </c>
+      <c r="D1764" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1764" t="inlineStr"/>
+      <c r="F1764" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g27</t>
+        </is>
+      </c>
+    </row>
+    <row r="1765">
+      <c r="A1765" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1765" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1765" t="inlineStr">
+        <is>
+          <t>PickingParts min</t>
+        </is>
+      </c>
+      <c r="D1765" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1765" t="inlineStr"/>
+      <c r="F1765" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g28</t>
+        </is>
+      </c>
+    </row>
+    <row r="1766">
+      <c r="A1766" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1766" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1766" t="inlineStr">
+        <is>
+          <t>PlacingParts min</t>
+        </is>
+      </c>
+      <c r="D1766" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1766" t="inlineStr"/>
+      <c r="F1766" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g29</t>
+        </is>
+      </c>
+    </row>
+    <row r="1767">
+      <c r="A1767" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1767" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1767" t="inlineStr">
+        <is>
+          <t>CountPickedReject14in</t>
+        </is>
+      </c>
+      <c r="D1767" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1767" t="inlineStr"/>
+      <c r="F1767" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1768">
+      <c r="A1768" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1768" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1768" t="inlineStr">
+        <is>
+          <t>temp_dsi</t>
+        </is>
+      </c>
+      <c r="D1768" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1768" t="inlineStr"/>
+      <c r="F1768" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g31</t>
+        </is>
+      </c>
+    </row>
+    <row r="1769">
+      <c r="A1769" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1769" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1769" t="inlineStr">
+        <is>
+          <t>temp_J1motor</t>
+        </is>
+      </c>
+      <c r="D1769" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1769" t="inlineStr"/>
+      <c r="F1769" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g32</t>
+        </is>
+      </c>
+    </row>
+    <row r="1770">
+      <c r="A1770" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1770" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1770" t="inlineStr">
+        <is>
+          <t>temp_J4motor</t>
+        </is>
+      </c>
+      <c r="D1770" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1770" t="inlineStr"/>
+      <c r="F1770" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g35</t>
+        </is>
+      </c>
+    </row>
+    <row r="1771">
+      <c r="A1771" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1771" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1771" t="inlineStr">
+        <is>
+          <t>temp_J6motor</t>
+        </is>
+      </c>
+      <c r="D1771" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1771" t="inlineStr"/>
+      <c r="F1771" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g37</t>
+        </is>
+      </c>
+    </row>
+    <row r="1772">
+      <c r="A1772" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1772" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1772" t="inlineStr">
+        <is>
+          <t>CountPickedRejectOTM</t>
+        </is>
+      </c>
+      <c r="D1772" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1772" t="inlineStr"/>
+      <c r="F1772" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g38</t>
+        </is>
+      </c>
+    </row>
+    <row r="1773">
+      <c r="A1773" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1773" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1773" t="inlineStr">
+        <is>
+          <t>CountPickedRejectPandral</t>
+        </is>
+      </c>
+      <c r="D1773" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1773" t="inlineStr"/>
+      <c r="F1773" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g39</t>
+        </is>
+      </c>
+    </row>
+    <row r="1774">
+      <c r="A1774" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1774" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1774" t="inlineStr">
+        <is>
+          <t>CountLaidButton</t>
+        </is>
+      </c>
+      <c r="D1774" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E1774" t="inlineStr"/>
+      <c r="F1774" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1775">
+      <c r="A1775" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1775" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1775" t="inlineStr">
+        <is>
+          <t>CountLaidDetector</t>
+        </is>
+      </c>
+      <c r="D1775" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1775" t="inlineStr"/>
+      <c r="F1775" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g3</t>
+        </is>
+      </c>
+    </row>
+    <row r="1776">
+      <c r="A1776" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1776" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1776" t="inlineStr">
+        <is>
+          <t>CountLaidEncoder</t>
+        </is>
+      </c>
+      <c r="D1776" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E1776" t="inlineStr"/>
+      <c r="F1776" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g4</t>
+        </is>
+      </c>
+    </row>
+    <row r="1777">
+      <c r="A1777" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1777" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1777" t="inlineStr">
+        <is>
+          <t>CountLaid14in</t>
+        </is>
+      </c>
+      <c r="D1777" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E1777" t="inlineStr"/>
+      <c r="F1777" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g5</t>
+        </is>
+      </c>
+    </row>
+    <row r="1778">
+      <c r="A1778" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1778" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1778" t="inlineStr">
+        <is>
+          <t>CountLaid18in</t>
+        </is>
+      </c>
+      <c r="D1778" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E1778" t="inlineStr"/>
+      <c r="F1778" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1779">
+      <c r="A1779" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1779" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1779" t="inlineStr">
+        <is>
+          <t>CountLaidPandral</t>
+        </is>
+      </c>
+      <c r="D1779" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1779" t="inlineStr"/>
+      <c r="F1779" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g7</t>
+        </is>
+      </c>
+    </row>
+    <row r="1780">
+      <c r="A1780" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1780" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1780" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D1780" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1780" t="inlineStr"/>
+      <c r="F1780" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g13</t>
+        </is>
+      </c>
+    </row>
+    <row r="1781">
+      <c r="A1781" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1781" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1781" t="inlineStr">
+        <is>
+          <t>CountAcceptedTotal</t>
+        </is>
+      </c>
+      <c r="D1781" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1781" t="inlineStr"/>
+      <c r="F1781" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g15</t>
+        </is>
+      </c>
+    </row>
+    <row r="1782">
+      <c r="A1782" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1782" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1782" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D1782" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1782" t="inlineStr"/>
+      <c r="F1782" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g17</t>
+        </is>
+      </c>
+    </row>
+    <row r="1783">
+      <c r="A1783" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1783" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1783" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D1783" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1783" t="inlineStr"/>
+      <c r="F1783" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g18</t>
+        </is>
+      </c>
+    </row>
+    <row r="1784">
+      <c r="A1784" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1784" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1784" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D1784" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1784" t="inlineStr"/>
+      <c r="F1784" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g19</t>
+        </is>
+      </c>
+    </row>
+    <row r="1785">
+      <c r="A1785" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1785" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1785" t="inlineStr">
+        <is>
+          <t>day_Servotime Hours10th</t>
+        </is>
+      </c>
+      <c r="D1785" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1785" t="inlineStr"/>
+      <c r="F1785" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g22</t>
+        </is>
+      </c>
+    </row>
+    <row r="1786">
+      <c r="A1786" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1786" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1786" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D1786" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1786" t="inlineStr"/>
+      <c r="F1786" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g23</t>
+        </is>
+      </c>
+    </row>
+    <row r="1787">
+      <c r="A1787" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1787" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1787" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D1787" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1787" t="inlineStr"/>
+      <c r="F1787" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g24</t>
+        </is>
+      </c>
+    </row>
+    <row r="1788">
+      <c r="A1788" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1788" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1788" t="inlineStr">
+        <is>
+          <t>tk_ClearPos</t>
+        </is>
+      </c>
+      <c r="D1788" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1788" t="inlineStr"/>
+      <c r="F1788" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g25</t>
+        </is>
+      </c>
+    </row>
+    <row r="1789">
+      <c r="A1789" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1789" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1789" t="inlineStr">
+        <is>
+          <t>temp_J2motor</t>
+        </is>
+      </c>
+      <c r="D1789" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1789" t="inlineStr"/>
+      <c r="F1789" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g33</t>
+        </is>
+      </c>
+    </row>
+    <row r="1790">
+      <c r="A1790" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1790" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1790" t="inlineStr">
+        <is>
+          <t>temp_J3motor</t>
+        </is>
+      </c>
+      <c r="D1790" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1790" t="inlineStr"/>
+      <c r="F1790" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g34</t>
+        </is>
+      </c>
+    </row>
+    <row r="1791">
+      <c r="A1791" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1791" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1791" t="inlineStr">
+        <is>
+          <t>temp_J5motor</t>
+        </is>
+      </c>
+      <c r="D1791" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1791" t="inlineStr"/>
+      <c r="F1791" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g36</t>
+        </is>
+      </c>
+    </row>
+    <row r="1792">
+      <c r="A1792" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:54:13</t>
+        </is>
+      </c>
+      <c r="B1792" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1792" t="inlineStr">
+        <is>
+          <t>CountPickedReject18in</t>
+        </is>
+      </c>
+      <c r="D1792" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1792" t="inlineStr"/>
+      <c r="F1792" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1793">
+      <c r="A1793" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:55:00</t>
+        </is>
+      </c>
+      <c r="B1793" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1793" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D1793" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1793" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1793" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1794">
+      <c r="A1794" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:55:00</t>
+        </is>
+      </c>
+      <c r="B1794" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1794" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D1794" t="b">
+        <v>1</v>
+      </c>
+      <c r="E1794" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1794" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1795">
+      <c r="A1795" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:55:00</t>
+        </is>
+      </c>
+      <c r="B1795" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1795" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D1795" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1795" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1795" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1796">
+      <c r="A1796" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:55:00</t>
+        </is>
+      </c>
+      <c r="B1796" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1796" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D1796" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1796" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1796" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1797">
+      <c r="A1797" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:55:00</t>
+        </is>
+      </c>
+      <c r="B1797" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1797" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D1797" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1797" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1797" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1798">
+      <c r="A1798" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:55:00</t>
+        </is>
+      </c>
+      <c r="B1798" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1798" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D1798" t="n">
+        <v>7925</v>
+      </c>
+      <c r="E1798" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1798" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1799">
+      <c r="A1799" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:55:00</t>
+        </is>
+      </c>
+      <c r="B1799" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1799" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D1799" t="n">
+        <v>2770</v>
+      </c>
+      <c r="E1799" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1799" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1800">
+      <c r="A1800" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:55:00</t>
+        </is>
+      </c>
+      <c r="B1800" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1800" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D1800" t="n">
+        <v>5155</v>
+      </c>
+      <c r="E1800" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1800" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1801">
+      <c r="A1801" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:55:00</t>
+        </is>
+      </c>
+      <c r="B1801" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1801" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D1801" t="n">
+        <v>0.6504731774330139</v>
+      </c>
+      <c r="E1801" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1801" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1802">
+      <c r="A1802" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:55:00</t>
+        </is>
+      </c>
+      <c r="B1802" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1802" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D1802" t="n">
+        <v>0.3495268225669861</v>
+      </c>
+      <c r="E1802" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1802" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1803">
+      <c r="A1803" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:55:00</t>
+        </is>
+      </c>
+      <c r="B1803" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1803" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D1803" t="n">
+        <v>1378</v>
+      </c>
+      <c r="E1803" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1803" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1804">
+      <c r="A1804" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:55:00</t>
+        </is>
+      </c>
+      <c r="B1804" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1804" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D1804" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1804" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1804" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1805">
+      <c r="A1805" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:55:00</t>
+        </is>
+      </c>
+      <c r="B1805" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1805" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D1805" t="n">
+        <v>1347</v>
+      </c>
+      <c r="E1805" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1805" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1806">
+      <c r="A1806" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:55:00</t>
+        </is>
+      </c>
+      <c r="B1806" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1806" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D1806" t="n">
+        <v>0.9775036573410034</v>
+      </c>
+      <c r="E1806" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1806" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1807">
+      <c r="A1807" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:55:00</t>
+        </is>
+      </c>
+      <c r="B1807" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1807" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D1807" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1807" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1807" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1808">
+      <c r="A1808" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:55:00</t>
+        </is>
+      </c>
+      <c r="B1808" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1808" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D1808" t="n">
+        <v>10.43280792236328</v>
+      </c>
+      <c r="E1808" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1808" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1809">
+      <c r="A1809" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:55:00</t>
+        </is>
+      </c>
+      <c r="B1809" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1809" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D1809" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1809" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1809" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1810">
+      <c r="A1810" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:55:00</t>
+        </is>
+      </c>
+      <c r="B1810" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1810" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D1810" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1810" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1810" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1811">
+      <c r="A1811" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:55:00</t>
+        </is>
+      </c>
+      <c r="B1811" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1811" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D1811" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1811" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1811" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1812">
+      <c r="A1812" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:55:00</t>
+        </is>
+      </c>
+      <c r="B1812" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1812" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D1812" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1812" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1812" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1813">
+      <c r="A1813" t="inlineStr">
+        <is>
+          <t>2026-08-17T15:55:00</t>
+        </is>
+      </c>
+      <c r="B1813" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1813" t="inlineStr">
+        <is>
+          <t>10thsInches_Tie Next</t>
+        </is>
+      </c>
+      <c r="D1813" t="n">
+        <v>195</v>
+      </c>
+      <c r="E1813" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1813" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/plc</t>
         </is>

</xml_diff>

<commit_message>
Log MQTT data 2026-08-17 17:01 UTC
</commit_message>
<xml_diff>
--- a/logs/raiv_tracker_2026-08-17.xlsx
+++ b/logs/raiv_tracker_2026-08-17.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1813"/>
+  <dimension ref="A1:F1913"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -48901,7 +48901,6 @@
           <t>13</t>
         </is>
       </c>
-      <c r="E1753" t="inlineStr"/>
       <c r="F1753" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g1</t>
@@ -48929,7 +48928,6 @@
           <t>1186</t>
         </is>
       </c>
-      <c r="E1754" t="inlineStr"/>
       <c r="F1754" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g8</t>
@@ -48957,7 +48955,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1755" t="inlineStr"/>
       <c r="F1755" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g9</t>
@@ -48985,7 +48982,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E1756" t="inlineStr"/>
       <c r="F1756" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g10</t>
@@ -49013,7 +49009,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E1757" t="inlineStr"/>
       <c r="F1757" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g11</t>
@@ -49041,7 +49036,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E1758" t="inlineStr"/>
       <c r="F1758" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g12</t>
@@ -49069,7 +49063,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1759" t="inlineStr"/>
       <c r="F1759" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g14</t>
@@ -49097,7 +49090,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1760" t="inlineStr"/>
       <c r="F1760" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g16</t>
@@ -49125,7 +49117,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1761" t="inlineStr"/>
       <c r="F1761" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g20</t>
@@ -49153,7 +49144,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1762" t="inlineStr"/>
       <c r="F1762" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g21</t>
@@ -49181,7 +49171,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1763" t="inlineStr"/>
       <c r="F1763" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g26</t>
@@ -49209,7 +49198,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1764" t="inlineStr"/>
       <c r="F1764" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g27</t>
@@ -49237,7 +49225,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1765" t="inlineStr"/>
       <c r="F1765" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g28</t>
@@ -49265,7 +49252,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1766" t="inlineStr"/>
       <c r="F1766" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g29</t>
@@ -49293,7 +49279,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1767" t="inlineStr"/>
       <c r="F1767" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g30</t>
@@ -49321,7 +49306,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1768" t="inlineStr"/>
       <c r="F1768" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g31</t>
@@ -49349,7 +49333,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1769" t="inlineStr"/>
       <c r="F1769" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g32</t>
@@ -49377,7 +49360,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1770" t="inlineStr"/>
       <c r="F1770" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g35</t>
@@ -49405,7 +49387,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1771" t="inlineStr"/>
       <c r="F1771" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g37</t>
@@ -49433,7 +49414,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1772" t="inlineStr"/>
       <c r="F1772" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g38</t>
@@ -49461,7 +49441,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1773" t="inlineStr"/>
       <c r="F1773" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g39</t>
@@ -49489,7 +49468,6 @@
           <t>6</t>
         </is>
       </c>
-      <c r="E1774" t="inlineStr"/>
       <c r="F1774" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g2</t>
@@ -49517,7 +49495,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1775" t="inlineStr"/>
       <c r="F1775" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g3</t>
@@ -49545,7 +49522,6 @@
           <t>7</t>
         </is>
       </c>
-      <c r="E1776" t="inlineStr"/>
       <c r="F1776" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g4</t>
@@ -49573,7 +49549,6 @@
           <t>11</t>
         </is>
       </c>
-      <c r="E1777" t="inlineStr"/>
       <c r="F1777" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g5</t>
@@ -49601,7 +49576,6 @@
           <t>2</t>
         </is>
       </c>
-      <c r="E1778" t="inlineStr"/>
       <c r="F1778" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g6</t>
@@ -49629,7 +49603,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1779" t="inlineStr"/>
       <c r="F1779" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g7</t>
@@ -49657,7 +49630,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1780" t="inlineStr"/>
       <c r="F1780" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g13</t>
@@ -49685,7 +49657,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1781" t="inlineStr"/>
       <c r="F1781" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g15</t>
@@ -49713,7 +49684,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1782" t="inlineStr"/>
       <c r="F1782" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g17</t>
@@ -49741,7 +49711,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1783" t="inlineStr"/>
       <c r="F1783" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g18</t>
@@ -49769,7 +49738,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1784" t="inlineStr"/>
       <c r="F1784" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g19</t>
@@ -49797,7 +49765,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1785" t="inlineStr"/>
       <c r="F1785" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g22</t>
@@ -49825,7 +49792,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1786" t="inlineStr"/>
       <c r="F1786" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g23</t>
@@ -49853,7 +49819,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1787" t="inlineStr"/>
       <c r="F1787" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g24</t>
@@ -49881,7 +49846,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1788" t="inlineStr"/>
       <c r="F1788" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g25</t>
@@ -49909,7 +49873,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1789" t="inlineStr"/>
       <c r="F1789" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g33</t>
@@ -49937,7 +49900,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1790" t="inlineStr"/>
       <c r="F1790" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g34</t>
@@ -49965,7 +49927,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1791" t="inlineStr"/>
       <c r="F1791" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g36</t>
@@ -49993,7 +49954,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1792" t="inlineStr"/>
       <c r="F1792" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g40</t>
@@ -50585,6 +50545,2806 @@
       <c r="F1813" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1814">
+      <c r="A1814" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1814" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1814" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D1814" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1814" t="inlineStr"/>
+      <c r="F1814" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1815">
+      <c r="A1815" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1815" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1815" t="inlineStr">
+        <is>
+          <t>CountLaidEncoder</t>
+        </is>
+      </c>
+      <c r="D1815" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1815" t="inlineStr"/>
+      <c r="F1815" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g4</t>
+        </is>
+      </c>
+    </row>
+    <row r="1816">
+      <c r="A1816" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1816" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1816" t="inlineStr">
+        <is>
+          <t>CountLaidButton</t>
+        </is>
+      </c>
+      <c r="D1816" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1816" t="inlineStr"/>
+      <c r="F1816" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1817">
+      <c r="A1817" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1817" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1817" t="inlineStr">
+        <is>
+          <t>CountLaidDetector</t>
+        </is>
+      </c>
+      <c r="D1817" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1817" t="inlineStr"/>
+      <c r="F1817" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g3</t>
+        </is>
+      </c>
+    </row>
+    <row r="1818">
+      <c r="A1818" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1818" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1818" t="inlineStr">
+        <is>
+          <t>CountLaid14in</t>
+        </is>
+      </c>
+      <c r="D1818" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1818" t="inlineStr"/>
+      <c r="F1818" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g5</t>
+        </is>
+      </c>
+    </row>
+    <row r="1819">
+      <c r="A1819" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1819" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1819" t="inlineStr">
+        <is>
+          <t>CountLaid18in</t>
+        </is>
+      </c>
+      <c r="D1819" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1819" t="inlineStr"/>
+      <c r="F1819" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1820">
+      <c r="A1820" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1820" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1820" t="inlineStr">
+        <is>
+          <t>CountLaidPandral</t>
+        </is>
+      </c>
+      <c r="D1820" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1820" t="inlineStr"/>
+      <c r="F1820" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g7</t>
+        </is>
+      </c>
+    </row>
+    <row r="1821">
+      <c r="A1821" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1821" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1821" t="inlineStr">
+        <is>
+          <t>usr_TPStime Hours10th</t>
+        </is>
+      </c>
+      <c r="D1821" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1821" t="inlineStr"/>
+      <c r="F1821" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g8</t>
+        </is>
+      </c>
+    </row>
+    <row r="1822">
+      <c r="A1822" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1822" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1822" t="inlineStr">
+        <is>
+          <t>usrTPS_miles xxx</t>
+        </is>
+      </c>
+      <c r="D1822" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1822" t="inlineStr"/>
+      <c r="F1822" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g9</t>
+        </is>
+      </c>
+    </row>
+    <row r="1823">
+      <c r="A1823" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1823" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1823" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D1823" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1823" t="inlineStr"/>
+      <c r="F1823" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g11</t>
+        </is>
+      </c>
+    </row>
+    <row r="1824">
+      <c r="A1824" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1824" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1824" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D1824" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E1824" t="inlineStr"/>
+      <c r="F1824" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g12</t>
+        </is>
+      </c>
+    </row>
+    <row r="1825">
+      <c r="A1825" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1825" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1825" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D1825" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1825" t="inlineStr"/>
+      <c r="F1825" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g13</t>
+        </is>
+      </c>
+    </row>
+    <row r="1826">
+      <c r="A1826" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1826" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1826" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D1826" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1826" t="inlineStr"/>
+      <c r="F1826" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g17</t>
+        </is>
+      </c>
+    </row>
+    <row r="1827">
+      <c r="A1827" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1827" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1827" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D1827" t="inlineStr">
+        <is>
+          <t>1378</t>
+        </is>
+      </c>
+      <c r="E1827" t="inlineStr"/>
+      <c r="F1827" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g18</t>
+        </is>
+      </c>
+    </row>
+    <row r="1828">
+      <c r="A1828" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1828" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1828" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D1828" t="inlineStr">
+        <is>
+          <t>1347</t>
+        </is>
+      </c>
+      <c r="E1828" t="inlineStr"/>
+      <c r="F1828" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g19</t>
+        </is>
+      </c>
+    </row>
+    <row r="1829">
+      <c r="A1829" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1829" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1829" t="inlineStr">
+        <is>
+          <t>tk_Cycle hrs</t>
+        </is>
+      </c>
+      <c r="D1829" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E1829" t="inlineStr"/>
+      <c r="F1829" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g21</t>
+        </is>
+      </c>
+    </row>
+    <row r="1830">
+      <c r="A1830" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1830" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1830" t="inlineStr">
+        <is>
+          <t>tk_ClearPos</t>
+        </is>
+      </c>
+      <c r="D1830" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1830" t="inlineStr"/>
+      <c r="F1830" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g25</t>
+        </is>
+      </c>
+    </row>
+    <row r="1831">
+      <c r="A1831" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1831" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1831" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D1831" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1831" t="inlineStr"/>
+      <c r="F1831" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g10</t>
+        </is>
+      </c>
+    </row>
+    <row r="1832">
+      <c r="A1832" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1832" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1832" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D1832" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1832" t="inlineStr"/>
+      <c r="F1832" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g14</t>
+        </is>
+      </c>
+    </row>
+    <row r="1833">
+      <c r="A1833" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1833" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1833" t="inlineStr">
+        <is>
+          <t>CountAcceptedTotal</t>
+        </is>
+      </c>
+      <c r="D1833" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1833" t="inlineStr"/>
+      <c r="F1833" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g15</t>
+        </is>
+      </c>
+    </row>
+    <row r="1834">
+      <c r="A1834" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1834" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1834" t="inlineStr">
+        <is>
+          <t>CountRejectedTotal</t>
+        </is>
+      </c>
+      <c r="D1834" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1834" t="inlineStr"/>
+      <c r="F1834" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g16</t>
+        </is>
+      </c>
+    </row>
+    <row r="1835">
+      <c r="A1835" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1835" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1835" t="inlineStr">
+        <is>
+          <t>day_Servotime Hours10th</t>
+        </is>
+      </c>
+      <c r="D1835" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="E1835" t="inlineStr"/>
+      <c r="F1835" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g22</t>
+        </is>
+      </c>
+    </row>
+    <row r="1836">
+      <c r="A1836" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1836" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1836" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D1836" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1836" t="inlineStr"/>
+      <c r="F1836" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g23</t>
+        </is>
+      </c>
+    </row>
+    <row r="1837">
+      <c r="A1837" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1837" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1837" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D1837" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1837" t="inlineStr"/>
+      <c r="F1837" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g24</t>
+        </is>
+      </c>
+    </row>
+    <row r="1838">
+      <c r="A1838" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1838" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1838" t="inlineStr">
+        <is>
+          <t>tk_Warmup</t>
+        </is>
+      </c>
+      <c r="D1838" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1838" t="inlineStr"/>
+      <c r="F1838" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g26</t>
+        </is>
+      </c>
+    </row>
+    <row r="1839">
+      <c r="A1839" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1839" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1839" t="inlineStr">
+        <is>
+          <t>FindingParts min</t>
+        </is>
+      </c>
+      <c r="D1839" t="inlineStr">
+        <is>
+          <t>147</t>
+        </is>
+      </c>
+      <c r="E1839" t="inlineStr"/>
+      <c r="F1839" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g27</t>
+        </is>
+      </c>
+    </row>
+    <row r="1840">
+      <c r="A1840" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1840" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1840" t="inlineStr">
+        <is>
+          <t>temp_dsi</t>
+        </is>
+      </c>
+      <c r="D1840" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1840" t="inlineStr"/>
+      <c r="F1840" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g31</t>
+        </is>
+      </c>
+    </row>
+    <row r="1841">
+      <c r="A1841" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1841" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1841" t="inlineStr">
+        <is>
+          <t>PickingParts min</t>
+        </is>
+      </c>
+      <c r="D1841" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="E1841" t="inlineStr"/>
+      <c r="F1841" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g28</t>
+        </is>
+      </c>
+    </row>
+    <row r="1842">
+      <c r="A1842" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1842" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1842" t="inlineStr">
+        <is>
+          <t>temp_J1motor</t>
+        </is>
+      </c>
+      <c r="D1842" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1842" t="inlineStr"/>
+      <c r="F1842" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g32</t>
+        </is>
+      </c>
+    </row>
+    <row r="1843">
+      <c r="A1843" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1843" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1843" t="inlineStr">
+        <is>
+          <t>temp_J2motor</t>
+        </is>
+      </c>
+      <c r="D1843" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1843" t="inlineStr"/>
+      <c r="F1843" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g33</t>
+        </is>
+      </c>
+    </row>
+    <row r="1844">
+      <c r="A1844" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1844" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1844" t="inlineStr">
+        <is>
+          <t>PlacingParts min</t>
+        </is>
+      </c>
+      <c r="D1844" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="E1844" t="inlineStr"/>
+      <c r="F1844" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g29</t>
+        </is>
+      </c>
+    </row>
+    <row r="1845">
+      <c r="A1845" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1845" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1845" t="inlineStr">
+        <is>
+          <t>CountPickedReject14in</t>
+        </is>
+      </c>
+      <c r="D1845" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1845" t="inlineStr"/>
+      <c r="F1845" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1846">
+      <c r="A1846" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1846" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1846" t="inlineStr">
+        <is>
+          <t>temp_J3motor</t>
+        </is>
+      </c>
+      <c r="D1846" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1846" t="inlineStr"/>
+      <c r="F1846" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g34</t>
+        </is>
+      </c>
+    </row>
+    <row r="1847">
+      <c r="A1847" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1847" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1847" t="inlineStr">
+        <is>
+          <t>temp_J4motor</t>
+        </is>
+      </c>
+      <c r="D1847" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1847" t="inlineStr"/>
+      <c r="F1847" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g35</t>
+        </is>
+      </c>
+    </row>
+    <row r="1848">
+      <c r="A1848" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1848" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1848" t="inlineStr">
+        <is>
+          <t>temp_J5motor</t>
+        </is>
+      </c>
+      <c r="D1848" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1848" t="inlineStr"/>
+      <c r="F1848" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g36</t>
+        </is>
+      </c>
+    </row>
+    <row r="1849">
+      <c r="A1849" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1849" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1849" t="inlineStr">
+        <is>
+          <t>CountPickedRejectOTM</t>
+        </is>
+      </c>
+      <c r="D1849" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1849" t="inlineStr"/>
+      <c r="F1849" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g38</t>
+        </is>
+      </c>
+    </row>
+    <row r="1850">
+      <c r="A1850" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1850" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1850" t="inlineStr">
+        <is>
+          <t>temp_J6motor</t>
+        </is>
+      </c>
+      <c r="D1850" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1850" t="inlineStr"/>
+      <c r="F1850" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g37</t>
+        </is>
+      </c>
+    </row>
+    <row r="1851">
+      <c r="A1851" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1851" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1851" t="inlineStr">
+        <is>
+          <t>CountPickedRejectPandral</t>
+        </is>
+      </c>
+      <c r="D1851" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1851" t="inlineStr"/>
+      <c r="F1851" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g39</t>
+        </is>
+      </c>
+    </row>
+    <row r="1852">
+      <c r="A1852" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:00:19</t>
+        </is>
+      </c>
+      <c r="B1852" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C1852" t="inlineStr">
+        <is>
+          <t>CountPickedReject18in</t>
+        </is>
+      </c>
+      <c r="D1852" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1852" t="inlineStr"/>
+      <c r="F1852" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1853">
+      <c r="A1853" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:00</t>
+        </is>
+      </c>
+      <c r="B1853" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1853" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D1853" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1853" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1853" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1854">
+      <c r="A1854" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:00</t>
+        </is>
+      </c>
+      <c r="B1854" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1854" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D1854" t="b">
+        <v>1</v>
+      </c>
+      <c r="E1854" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1854" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1855">
+      <c r="A1855" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:00</t>
+        </is>
+      </c>
+      <c r="B1855" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1855" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D1855" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1855" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1855" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1856">
+      <c r="A1856" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:00</t>
+        </is>
+      </c>
+      <c r="B1856" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1856" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D1856" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1856" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1856" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1857">
+      <c r="A1857" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:00</t>
+        </is>
+      </c>
+      <c r="B1857" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1857" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D1857" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1857" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1857" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1858">
+      <c r="A1858" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:00</t>
+        </is>
+      </c>
+      <c r="B1858" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1858" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D1858" t="n">
+        <v>7925</v>
+      </c>
+      <c r="E1858" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1858" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1859">
+      <c r="A1859" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:00</t>
+        </is>
+      </c>
+      <c r="B1859" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1859" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D1859" t="n">
+        <v>2770</v>
+      </c>
+      <c r="E1859" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1859" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1860">
+      <c r="A1860" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:00</t>
+        </is>
+      </c>
+      <c r="B1860" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1860" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D1860" t="n">
+        <v>5155</v>
+      </c>
+      <c r="E1860" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1860" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1861">
+      <c r="A1861" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:00</t>
+        </is>
+      </c>
+      <c r="B1861" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1861" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D1861" t="n">
+        <v>0.6504731774330139</v>
+      </c>
+      <c r="E1861" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1861" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1862">
+      <c r="A1862" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:00</t>
+        </is>
+      </c>
+      <c r="B1862" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1862" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D1862" t="n">
+        <v>0.3495268225669861</v>
+      </c>
+      <c r="E1862" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1862" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1863">
+      <c r="A1863" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:00</t>
+        </is>
+      </c>
+      <c r="B1863" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1863" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D1863" t="n">
+        <v>1378</v>
+      </c>
+      <c r="E1863" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1863" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1864">
+      <c r="A1864" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:00</t>
+        </is>
+      </c>
+      <c r="B1864" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1864" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D1864" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1864" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1864" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1865">
+      <c r="A1865" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:00</t>
+        </is>
+      </c>
+      <c r="B1865" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1865" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D1865" t="n">
+        <v>1347</v>
+      </c>
+      <c r="E1865" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1865" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1866">
+      <c r="A1866" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:00</t>
+        </is>
+      </c>
+      <c r="B1866" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1866" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D1866" t="n">
+        <v>0.9775036573410034</v>
+      </c>
+      <c r="E1866" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1866" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1867">
+      <c r="A1867" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:00</t>
+        </is>
+      </c>
+      <c r="B1867" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1867" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D1867" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1867" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1867" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1868">
+      <c r="A1868" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:00</t>
+        </is>
+      </c>
+      <c r="B1868" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1868" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D1868" t="n">
+        <v>10.43280792236328</v>
+      </c>
+      <c r="E1868" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1868" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1869">
+      <c r="A1869" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:00</t>
+        </is>
+      </c>
+      <c r="B1869" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1869" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D1869" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1869" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1869" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1870">
+      <c r="A1870" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:00</t>
+        </is>
+      </c>
+      <c r="B1870" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1870" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D1870" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1870" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1870" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1871">
+      <c r="A1871" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:00</t>
+        </is>
+      </c>
+      <c r="B1871" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1871" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D1871" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1871" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1871" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1872">
+      <c r="A1872" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:00</t>
+        </is>
+      </c>
+      <c r="B1872" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1872" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D1872" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1872" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1872" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1873">
+      <c r="A1873" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:00</t>
+        </is>
+      </c>
+      <c r="B1873" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1873" t="inlineStr">
+        <is>
+          <t>10thsInches_Tie Next</t>
+        </is>
+      </c>
+      <c r="D1873" t="n">
+        <v>195</v>
+      </c>
+      <c r="E1873" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1873" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1874">
+      <c r="A1874" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1874" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1874" t="inlineStr">
+        <is>
+          <t>CountLaidButton</t>
+        </is>
+      </c>
+      <c r="D1874" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E1874" t="inlineStr"/>
+      <c r="F1874" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1875">
+      <c r="A1875" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1875" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1875" t="inlineStr">
+        <is>
+          <t>CountLaidDetector</t>
+        </is>
+      </c>
+      <c r="D1875" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1875" t="inlineStr"/>
+      <c r="F1875" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g3</t>
+        </is>
+      </c>
+    </row>
+    <row r="1876">
+      <c r="A1876" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1876" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1876" t="inlineStr">
+        <is>
+          <t>CountLaidEncoder</t>
+        </is>
+      </c>
+      <c r="D1876" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E1876" t="inlineStr"/>
+      <c r="F1876" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g4</t>
+        </is>
+      </c>
+    </row>
+    <row r="1877">
+      <c r="A1877" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1877" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1877" t="inlineStr">
+        <is>
+          <t>CountLaid14in</t>
+        </is>
+      </c>
+      <c r="D1877" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E1877" t="inlineStr"/>
+      <c r="F1877" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g5</t>
+        </is>
+      </c>
+    </row>
+    <row r="1878">
+      <c r="A1878" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1878" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1878" t="inlineStr">
+        <is>
+          <t>CountLaid18in</t>
+        </is>
+      </c>
+      <c r="D1878" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E1878" t="inlineStr"/>
+      <c r="F1878" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1879">
+      <c r="A1879" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1879" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1879" t="inlineStr">
+        <is>
+          <t>CountLaidPandral</t>
+        </is>
+      </c>
+      <c r="D1879" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1879" t="inlineStr"/>
+      <c r="F1879" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g7</t>
+        </is>
+      </c>
+    </row>
+    <row r="1880">
+      <c r="A1880" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1880" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1880" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D1880" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E1880" t="inlineStr"/>
+      <c r="F1880" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1881">
+      <c r="A1881" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1881" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1881" t="inlineStr">
+        <is>
+          <t>usr_TPStime Hours10th</t>
+        </is>
+      </c>
+      <c r="D1881" t="inlineStr">
+        <is>
+          <t>1197</t>
+        </is>
+      </c>
+      <c r="E1881" t="inlineStr"/>
+      <c r="F1881" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g8</t>
+        </is>
+      </c>
+    </row>
+    <row r="1882">
+      <c r="A1882" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1882" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1882" t="inlineStr">
+        <is>
+          <t>usrTPS_miles xxx</t>
+        </is>
+      </c>
+      <c r="D1882" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1882" t="inlineStr"/>
+      <c r="F1882" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g9</t>
+        </is>
+      </c>
+    </row>
+    <row r="1883">
+      <c r="A1883" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1883" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1883" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D1883" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E1883" t="inlineStr"/>
+      <c r="F1883" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g10</t>
+        </is>
+      </c>
+    </row>
+    <row r="1884">
+      <c r="A1884" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1884" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1884" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D1884" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E1884" t="inlineStr"/>
+      <c r="F1884" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g11</t>
+        </is>
+      </c>
+    </row>
+    <row r="1885">
+      <c r="A1885" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1885" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1885" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D1885" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E1885" t="inlineStr"/>
+      <c r="F1885" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g12</t>
+        </is>
+      </c>
+    </row>
+    <row r="1886">
+      <c r="A1886" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1886" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1886" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D1886" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1886" t="inlineStr"/>
+      <c r="F1886" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g13</t>
+        </is>
+      </c>
+    </row>
+    <row r="1887">
+      <c r="A1887" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1887" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1887" t="inlineStr">
+        <is>
+          <t>CountAcceptedTotal</t>
+        </is>
+      </c>
+      <c r="D1887" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1887" t="inlineStr"/>
+      <c r="F1887" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g15</t>
+        </is>
+      </c>
+    </row>
+    <row r="1888">
+      <c r="A1888" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1888" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1888" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D1888" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1888" t="inlineStr"/>
+      <c r="F1888" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g17</t>
+        </is>
+      </c>
+    </row>
+    <row r="1889">
+      <c r="A1889" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1889" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1889" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D1889" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1889" t="inlineStr"/>
+      <c r="F1889" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g18</t>
+        </is>
+      </c>
+    </row>
+    <row r="1890">
+      <c r="A1890" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1890" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1890" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D1890" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1890" t="inlineStr"/>
+      <c r="F1890" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g19</t>
+        </is>
+      </c>
+    </row>
+    <row r="1891">
+      <c r="A1891" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1891" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1891" t="inlineStr">
+        <is>
+          <t>day_Servotime Hours10th</t>
+        </is>
+      </c>
+      <c r="D1891" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1891" t="inlineStr"/>
+      <c r="F1891" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g22</t>
+        </is>
+      </c>
+    </row>
+    <row r="1892">
+      <c r="A1892" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1892" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1892" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D1892" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1892" t="inlineStr"/>
+      <c r="F1892" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g23</t>
+        </is>
+      </c>
+    </row>
+    <row r="1893">
+      <c r="A1893" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1893" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1893" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D1893" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1893" t="inlineStr"/>
+      <c r="F1893" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g24</t>
+        </is>
+      </c>
+    </row>
+    <row r="1894">
+      <c r="A1894" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1894" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1894" t="inlineStr">
+        <is>
+          <t>tk_ClearPos</t>
+        </is>
+      </c>
+      <c r="D1894" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1894" t="inlineStr"/>
+      <c r="F1894" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g25</t>
+        </is>
+      </c>
+    </row>
+    <row r="1895">
+      <c r="A1895" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1895" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1895" t="inlineStr">
+        <is>
+          <t>temp_J2motor</t>
+        </is>
+      </c>
+      <c r="D1895" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1895" t="inlineStr"/>
+      <c r="F1895" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g33</t>
+        </is>
+      </c>
+    </row>
+    <row r="1896">
+      <c r="A1896" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1896" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1896" t="inlineStr">
+        <is>
+          <t>temp_J3motor</t>
+        </is>
+      </c>
+      <c r="D1896" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1896" t="inlineStr"/>
+      <c r="F1896" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g34</t>
+        </is>
+      </c>
+    </row>
+    <row r="1897">
+      <c r="A1897" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1897" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1897" t="inlineStr">
+        <is>
+          <t>temp_J5motor</t>
+        </is>
+      </c>
+      <c r="D1897" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1897" t="inlineStr"/>
+      <c r="F1897" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g36</t>
+        </is>
+      </c>
+    </row>
+    <row r="1898">
+      <c r="A1898" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1898" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1898" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D1898" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1898" t="inlineStr"/>
+      <c r="F1898" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g14</t>
+        </is>
+      </c>
+    </row>
+    <row r="1899">
+      <c r="A1899" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1899" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1899" t="inlineStr">
+        <is>
+          <t>CountRejectedTotal</t>
+        </is>
+      </c>
+      <c r="D1899" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1899" t="inlineStr"/>
+      <c r="F1899" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g16</t>
+        </is>
+      </c>
+    </row>
+    <row r="1900">
+      <c r="A1900" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1900" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1900" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D1900" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1900" t="inlineStr"/>
+      <c r="F1900" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g20</t>
+        </is>
+      </c>
+    </row>
+    <row r="1901">
+      <c r="A1901" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1901" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1901" t="inlineStr">
+        <is>
+          <t>tk_Cycle hrs</t>
+        </is>
+      </c>
+      <c r="D1901" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1901" t="inlineStr"/>
+      <c r="F1901" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g21</t>
+        </is>
+      </c>
+    </row>
+    <row r="1902">
+      <c r="A1902" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1902" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1902" t="inlineStr">
+        <is>
+          <t>tk_Warmup</t>
+        </is>
+      </c>
+      <c r="D1902" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1902" t="inlineStr"/>
+      <c r="F1902" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g26</t>
+        </is>
+      </c>
+    </row>
+    <row r="1903">
+      <c r="A1903" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1903" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1903" t="inlineStr">
+        <is>
+          <t>FindingParts min</t>
+        </is>
+      </c>
+      <c r="D1903" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1903" t="inlineStr"/>
+      <c r="F1903" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g27</t>
+        </is>
+      </c>
+    </row>
+    <row r="1904">
+      <c r="A1904" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1904" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1904" t="inlineStr">
+        <is>
+          <t>PickingParts min</t>
+        </is>
+      </c>
+      <c r="D1904" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1904" t="inlineStr"/>
+      <c r="F1904" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g28</t>
+        </is>
+      </c>
+    </row>
+    <row r="1905">
+      <c r="A1905" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1905" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1905" t="inlineStr">
+        <is>
+          <t>PlacingParts min</t>
+        </is>
+      </c>
+      <c r="D1905" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1905" t="inlineStr"/>
+      <c r="F1905" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g29</t>
+        </is>
+      </c>
+    </row>
+    <row r="1906">
+      <c r="A1906" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1906" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1906" t="inlineStr">
+        <is>
+          <t>CountPickedReject14in</t>
+        </is>
+      </c>
+      <c r="D1906" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1906" t="inlineStr"/>
+      <c r="F1906" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1907">
+      <c r="A1907" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1907" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1907" t="inlineStr">
+        <is>
+          <t>temp_dsi</t>
+        </is>
+      </c>
+      <c r="D1907" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1907" t="inlineStr"/>
+      <c r="F1907" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g31</t>
+        </is>
+      </c>
+    </row>
+    <row r="1908">
+      <c r="A1908" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1908" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1908" t="inlineStr">
+        <is>
+          <t>temp_J1motor</t>
+        </is>
+      </c>
+      <c r="D1908" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1908" t="inlineStr"/>
+      <c r="F1908" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g32</t>
+        </is>
+      </c>
+    </row>
+    <row r="1909">
+      <c r="A1909" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1909" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1909" t="inlineStr">
+        <is>
+          <t>temp_J4motor</t>
+        </is>
+      </c>
+      <c r="D1909" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1909" t="inlineStr"/>
+      <c r="F1909" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g35</t>
+        </is>
+      </c>
+    </row>
+    <row r="1910">
+      <c r="A1910" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1910" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1910" t="inlineStr">
+        <is>
+          <t>temp_J6motor</t>
+        </is>
+      </c>
+      <c r="D1910" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1910" t="inlineStr"/>
+      <c r="F1910" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g37</t>
+        </is>
+      </c>
+    </row>
+    <row r="1911">
+      <c r="A1911" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1911" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1911" t="inlineStr">
+        <is>
+          <t>CountPickedRejectOTM</t>
+        </is>
+      </c>
+      <c r="D1911" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1911" t="inlineStr"/>
+      <c r="F1911" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g38</t>
+        </is>
+      </c>
+    </row>
+    <row r="1912">
+      <c r="A1912" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1912" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1912" t="inlineStr">
+        <is>
+          <t>CountPickedRejectPandral</t>
+        </is>
+      </c>
+      <c r="D1912" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1912" t="inlineStr"/>
+      <c r="F1912" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g39</t>
+        </is>
+      </c>
+    </row>
+    <row r="1913">
+      <c r="A1913" t="inlineStr">
+        <is>
+          <t>2026-08-17T17:01:13</t>
+        </is>
+      </c>
+      <c r="B1913" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1913" t="inlineStr">
+        <is>
+          <t>CountPickedReject18in</t>
+        </is>
+      </c>
+      <c r="D1913" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1913" t="inlineStr"/>
+      <c r="F1913" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log MQTT data 2026-08-17 18:05 UTC
</commit_message>
<xml_diff>
--- a/logs/raiv_tracker_2026-08-17.xlsx
+++ b/logs/raiv_tracker_2026-08-17.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1913"/>
+  <dimension ref="A1:F1953"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50569,7 +50569,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1814" t="inlineStr"/>
       <c r="F1814" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g1</t>
@@ -50597,7 +50596,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1815" t="inlineStr"/>
       <c r="F1815" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g4</t>
@@ -50625,7 +50623,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1816" t="inlineStr"/>
       <c r="F1816" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g2</t>
@@ -50653,7 +50650,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1817" t="inlineStr"/>
       <c r="F1817" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g3</t>
@@ -50681,7 +50677,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1818" t="inlineStr"/>
       <c r="F1818" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g5</t>
@@ -50709,7 +50704,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1819" t="inlineStr"/>
       <c r="F1819" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g6</t>
@@ -50737,7 +50731,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1820" t="inlineStr"/>
       <c r="F1820" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g7</t>
@@ -50765,7 +50758,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1821" t="inlineStr"/>
       <c r="F1821" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g8</t>
@@ -50793,7 +50785,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1822" t="inlineStr"/>
       <c r="F1822" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g9</t>
@@ -50821,7 +50812,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1823" t="inlineStr"/>
       <c r="F1823" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g11</t>
@@ -50849,7 +50839,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E1824" t="inlineStr"/>
       <c r="F1824" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g12</t>
@@ -50877,7 +50866,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1825" t="inlineStr"/>
       <c r="F1825" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g13</t>
@@ -50905,7 +50893,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1826" t="inlineStr"/>
       <c r="F1826" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g17</t>
@@ -50933,7 +50920,6 @@
           <t>1378</t>
         </is>
       </c>
-      <c r="E1827" t="inlineStr"/>
       <c r="F1827" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g18</t>
@@ -50961,7 +50947,6 @@
           <t>1347</t>
         </is>
       </c>
-      <c r="E1828" t="inlineStr"/>
       <c r="F1828" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g19</t>
@@ -50989,7 +50974,6 @@
           <t>6</t>
         </is>
       </c>
-      <c r="E1829" t="inlineStr"/>
       <c r="F1829" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g21</t>
@@ -51017,7 +51001,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1830" t="inlineStr"/>
       <c r="F1830" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g25</t>
@@ -51045,7 +51028,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1831" t="inlineStr"/>
       <c r="F1831" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g10</t>
@@ -51073,7 +51055,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1832" t="inlineStr"/>
       <c r="F1832" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g14</t>
@@ -51101,7 +51082,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1833" t="inlineStr"/>
       <c r="F1833" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g15</t>
@@ -51129,7 +51109,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1834" t="inlineStr"/>
       <c r="F1834" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g16</t>
@@ -51157,7 +51136,6 @@
           <t>22</t>
         </is>
       </c>
-      <c r="E1835" t="inlineStr"/>
       <c r="F1835" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g22</t>
@@ -51185,7 +51163,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1836" t="inlineStr"/>
       <c r="F1836" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g23</t>
@@ -51213,7 +51190,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1837" t="inlineStr"/>
       <c r="F1837" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g24</t>
@@ -51241,7 +51217,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1838" t="inlineStr"/>
       <c r="F1838" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g26</t>
@@ -51269,7 +51244,6 @@
           <t>147</t>
         </is>
       </c>
-      <c r="E1839" t="inlineStr"/>
       <c r="F1839" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g27</t>
@@ -51297,7 +51271,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1840" t="inlineStr"/>
       <c r="F1840" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g31</t>
@@ -51325,7 +51298,6 @@
           <t>41</t>
         </is>
       </c>
-      <c r="E1841" t="inlineStr"/>
       <c r="F1841" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g28</t>
@@ -51353,7 +51325,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1842" t="inlineStr"/>
       <c r="F1842" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g32</t>
@@ -51381,7 +51352,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1843" t="inlineStr"/>
       <c r="F1843" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g33</t>
@@ -51409,7 +51379,6 @@
           <t>43</t>
         </is>
       </c>
-      <c r="E1844" t="inlineStr"/>
       <c r="F1844" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g29</t>
@@ -51437,7 +51406,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1845" t="inlineStr"/>
       <c r="F1845" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g30</t>
@@ -51465,7 +51433,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1846" t="inlineStr"/>
       <c r="F1846" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g34</t>
@@ -51493,7 +51460,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1847" t="inlineStr"/>
       <c r="F1847" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g35</t>
@@ -51521,7 +51487,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1848" t="inlineStr"/>
       <c r="F1848" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g36</t>
@@ -51549,7 +51514,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1849" t="inlineStr"/>
       <c r="F1849" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g38</t>
@@ -51577,7 +51541,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1850" t="inlineStr"/>
       <c r="F1850" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g37</t>
@@ -51605,7 +51568,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1851" t="inlineStr"/>
       <c r="F1851" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g39</t>
@@ -51633,7 +51595,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1852" t="inlineStr"/>
       <c r="F1852" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g40</t>
@@ -52249,7 +52210,6 @@
           <t>6</t>
         </is>
       </c>
-      <c r="E1874" t="inlineStr"/>
       <c r="F1874" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g2</t>
@@ -52277,7 +52237,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1875" t="inlineStr"/>
       <c r="F1875" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g3</t>
@@ -52305,7 +52264,6 @@
           <t>7</t>
         </is>
       </c>
-      <c r="E1876" t="inlineStr"/>
       <c r="F1876" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g4</t>
@@ -52333,7 +52291,6 @@
           <t>11</t>
         </is>
       </c>
-      <c r="E1877" t="inlineStr"/>
       <c r="F1877" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g5</t>
@@ -52361,7 +52318,6 @@
           <t>2</t>
         </is>
       </c>
-      <c r="E1878" t="inlineStr"/>
       <c r="F1878" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g6</t>
@@ -52389,7 +52345,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1879" t="inlineStr"/>
       <c r="F1879" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g7</t>
@@ -52417,7 +52372,6 @@
           <t>13</t>
         </is>
       </c>
-      <c r="E1880" t="inlineStr"/>
       <c r="F1880" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g1</t>
@@ -52445,7 +52399,6 @@
           <t>1197</t>
         </is>
       </c>
-      <c r="E1881" t="inlineStr"/>
       <c r="F1881" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g8</t>
@@ -52473,7 +52426,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1882" t="inlineStr"/>
       <c r="F1882" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g9</t>
@@ -52501,7 +52453,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E1883" t="inlineStr"/>
       <c r="F1883" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g10</t>
@@ -52529,7 +52480,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E1884" t="inlineStr"/>
       <c r="F1884" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g11</t>
@@ -52557,7 +52507,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E1885" t="inlineStr"/>
       <c r="F1885" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g12</t>
@@ -52585,7 +52534,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1886" t="inlineStr"/>
       <c r="F1886" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g13</t>
@@ -52613,7 +52561,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1887" t="inlineStr"/>
       <c r="F1887" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g15</t>
@@ -52641,7 +52588,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1888" t="inlineStr"/>
       <c r="F1888" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g17</t>
@@ -52669,7 +52615,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1889" t="inlineStr"/>
       <c r="F1889" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g18</t>
@@ -52697,7 +52642,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1890" t="inlineStr"/>
       <c r="F1890" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g19</t>
@@ -52725,7 +52669,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1891" t="inlineStr"/>
       <c r="F1891" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g22</t>
@@ -52753,7 +52696,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1892" t="inlineStr"/>
       <c r="F1892" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g23</t>
@@ -52781,7 +52723,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1893" t="inlineStr"/>
       <c r="F1893" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g24</t>
@@ -52809,7 +52750,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1894" t="inlineStr"/>
       <c r="F1894" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g25</t>
@@ -52837,7 +52777,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1895" t="inlineStr"/>
       <c r="F1895" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g33</t>
@@ -52865,7 +52804,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1896" t="inlineStr"/>
       <c r="F1896" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g34</t>
@@ -52893,7 +52831,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1897" t="inlineStr"/>
       <c r="F1897" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g36</t>
@@ -52921,7 +52858,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1898" t="inlineStr"/>
       <c r="F1898" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g14</t>
@@ -52949,7 +52885,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1899" t="inlineStr"/>
       <c r="F1899" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g16</t>
@@ -52977,7 +52912,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1900" t="inlineStr"/>
       <c r="F1900" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g20</t>
@@ -53005,7 +52939,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1901" t="inlineStr"/>
       <c r="F1901" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g21</t>
@@ -53033,7 +52966,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1902" t="inlineStr"/>
       <c r="F1902" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g26</t>
@@ -53061,7 +52993,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1903" t="inlineStr"/>
       <c r="F1903" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g27</t>
@@ -53089,7 +53020,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1904" t="inlineStr"/>
       <c r="F1904" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g28</t>
@@ -53117,7 +53047,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1905" t="inlineStr"/>
       <c r="F1905" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g29</t>
@@ -53145,7 +53074,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1906" t="inlineStr"/>
       <c r="F1906" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g30</t>
@@ -53173,7 +53101,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1907" t="inlineStr"/>
       <c r="F1907" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g31</t>
@@ -53201,7 +53128,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1908" t="inlineStr"/>
       <c r="F1908" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g32</t>
@@ -53229,7 +53155,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1909" t="inlineStr"/>
       <c r="F1909" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g35</t>
@@ -53257,7 +53182,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1910" t="inlineStr"/>
       <c r="F1910" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g37</t>
@@ -53285,7 +53209,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1911" t="inlineStr"/>
       <c r="F1911" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g38</t>
@@ -53313,7 +53236,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1912" t="inlineStr"/>
       <c r="F1912" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g39</t>
@@ -53341,10 +53263,1129 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1913" t="inlineStr"/>
       <c r="F1913" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1914">
+      <c r="A1914" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1914" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1914" t="inlineStr">
+        <is>
+          <t>CountLaidButton</t>
+        </is>
+      </c>
+      <c r="D1914" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E1914" t="inlineStr"/>
+      <c r="F1914" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1915">
+      <c r="A1915" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1915" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1915" t="inlineStr">
+        <is>
+          <t>CountLaidDetector</t>
+        </is>
+      </c>
+      <c r="D1915" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1915" t="inlineStr"/>
+      <c r="F1915" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g3</t>
+        </is>
+      </c>
+    </row>
+    <row r="1916">
+      <c r="A1916" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1916" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1916" t="inlineStr">
+        <is>
+          <t>CountLaidEncoder</t>
+        </is>
+      </c>
+      <c r="D1916" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E1916" t="inlineStr"/>
+      <c r="F1916" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g4</t>
+        </is>
+      </c>
+    </row>
+    <row r="1917">
+      <c r="A1917" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1917" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1917" t="inlineStr">
+        <is>
+          <t>CountLaid14in</t>
+        </is>
+      </c>
+      <c r="D1917" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E1917" t="inlineStr"/>
+      <c r="F1917" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g5</t>
+        </is>
+      </c>
+    </row>
+    <row r="1918">
+      <c r="A1918" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1918" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1918" t="inlineStr">
+        <is>
+          <t>CountLaid18in</t>
+        </is>
+      </c>
+      <c r="D1918" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E1918" t="inlineStr"/>
+      <c r="F1918" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1919">
+      <c r="A1919" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1919" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1919" t="inlineStr">
+        <is>
+          <t>CountLaidPandral</t>
+        </is>
+      </c>
+      <c r="D1919" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1919" t="inlineStr"/>
+      <c r="F1919" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g7</t>
+        </is>
+      </c>
+    </row>
+    <row r="1920">
+      <c r="A1920" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1920" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1920" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D1920" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1920" t="inlineStr"/>
+      <c r="F1920" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g13</t>
+        </is>
+      </c>
+    </row>
+    <row r="1921">
+      <c r="A1921" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1921" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1921" t="inlineStr">
+        <is>
+          <t>CountAcceptedTotal</t>
+        </is>
+      </c>
+      <c r="D1921" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1921" t="inlineStr"/>
+      <c r="F1921" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g15</t>
+        </is>
+      </c>
+    </row>
+    <row r="1922">
+      <c r="A1922" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1922" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1922" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D1922" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1922" t="inlineStr"/>
+      <c r="F1922" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g17</t>
+        </is>
+      </c>
+    </row>
+    <row r="1923">
+      <c r="A1923" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1923" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1923" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D1923" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1923" t="inlineStr"/>
+      <c r="F1923" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g18</t>
+        </is>
+      </c>
+    </row>
+    <row r="1924">
+      <c r="A1924" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1924" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1924" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D1924" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1924" t="inlineStr"/>
+      <c r="F1924" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g19</t>
+        </is>
+      </c>
+    </row>
+    <row r="1925">
+      <c r="A1925" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1925" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1925" t="inlineStr">
+        <is>
+          <t>day_Servotime Hours10th</t>
+        </is>
+      </c>
+      <c r="D1925" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1925" t="inlineStr"/>
+      <c r="F1925" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g22</t>
+        </is>
+      </c>
+    </row>
+    <row r="1926">
+      <c r="A1926" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1926" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1926" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D1926" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1926" t="inlineStr"/>
+      <c r="F1926" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g23</t>
+        </is>
+      </c>
+    </row>
+    <row r="1927">
+      <c r="A1927" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1927" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1927" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D1927" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1927" t="inlineStr"/>
+      <c r="F1927" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g24</t>
+        </is>
+      </c>
+    </row>
+    <row r="1928">
+      <c r="A1928" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1928" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1928" t="inlineStr">
+        <is>
+          <t>tk_ClearPos</t>
+        </is>
+      </c>
+      <c r="D1928" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1928" t="inlineStr"/>
+      <c r="F1928" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g25</t>
+        </is>
+      </c>
+    </row>
+    <row r="1929">
+      <c r="A1929" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1929" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1929" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D1929" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E1929" t="inlineStr"/>
+      <c r="F1929" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1930">
+      <c r="A1930" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1930" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1930" t="inlineStr">
+        <is>
+          <t>temp_J2motor</t>
+        </is>
+      </c>
+      <c r="D1930" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1930" t="inlineStr"/>
+      <c r="F1930" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g33</t>
+        </is>
+      </c>
+    </row>
+    <row r="1931">
+      <c r="A1931" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1931" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1931" t="inlineStr">
+        <is>
+          <t>temp_J3motor</t>
+        </is>
+      </c>
+      <c r="D1931" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1931" t="inlineStr"/>
+      <c r="F1931" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g34</t>
+        </is>
+      </c>
+    </row>
+    <row r="1932">
+      <c r="A1932" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1932" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1932" t="inlineStr">
+        <is>
+          <t>usr_TPStime Hours10th</t>
+        </is>
+      </c>
+      <c r="D1932" t="inlineStr">
+        <is>
+          <t>1208</t>
+        </is>
+      </c>
+      <c r="E1932" t="inlineStr"/>
+      <c r="F1932" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g8</t>
+        </is>
+      </c>
+    </row>
+    <row r="1933">
+      <c r="A1933" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1933" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1933" t="inlineStr">
+        <is>
+          <t>usrTPS_miles xxx</t>
+        </is>
+      </c>
+      <c r="D1933" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1933" t="inlineStr"/>
+      <c r="F1933" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g9</t>
+        </is>
+      </c>
+    </row>
+    <row r="1934">
+      <c r="A1934" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1934" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1934" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D1934" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E1934" t="inlineStr"/>
+      <c r="F1934" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g10</t>
+        </is>
+      </c>
+    </row>
+    <row r="1935">
+      <c r="A1935" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1935" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1935" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D1935" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E1935" t="inlineStr"/>
+      <c r="F1935" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g11</t>
+        </is>
+      </c>
+    </row>
+    <row r="1936">
+      <c r="A1936" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1936" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1936" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D1936" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E1936" t="inlineStr"/>
+      <c r="F1936" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g12</t>
+        </is>
+      </c>
+    </row>
+    <row r="1937">
+      <c r="A1937" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1937" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1937" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D1937" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1937" t="inlineStr"/>
+      <c r="F1937" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g14</t>
+        </is>
+      </c>
+    </row>
+    <row r="1938">
+      <c r="A1938" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1938" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1938" t="inlineStr">
+        <is>
+          <t>CountRejectedTotal</t>
+        </is>
+      </c>
+      <c r="D1938" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1938" t="inlineStr"/>
+      <c r="F1938" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g16</t>
+        </is>
+      </c>
+    </row>
+    <row r="1939">
+      <c r="A1939" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1939" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1939" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D1939" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1939" t="inlineStr"/>
+      <c r="F1939" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g20</t>
+        </is>
+      </c>
+    </row>
+    <row r="1940">
+      <c r="A1940" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1940" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1940" t="inlineStr">
+        <is>
+          <t>tk_Cycle hrs</t>
+        </is>
+      </c>
+      <c r="D1940" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1940" t="inlineStr"/>
+      <c r="F1940" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g21</t>
+        </is>
+      </c>
+    </row>
+    <row r="1941">
+      <c r="A1941" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1941" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1941" t="inlineStr">
+        <is>
+          <t>temp_J5motor</t>
+        </is>
+      </c>
+      <c r="D1941" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1941" t="inlineStr"/>
+      <c r="F1941" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g36</t>
+        </is>
+      </c>
+    </row>
+    <row r="1942">
+      <c r="A1942" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1942" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1942" t="inlineStr">
+        <is>
+          <t>CountPickedReject18in</t>
+        </is>
+      </c>
+      <c r="D1942" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1942" t="inlineStr"/>
+      <c r="F1942" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1943">
+      <c r="A1943" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1943" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1943" t="inlineStr">
+        <is>
+          <t>tk_Warmup</t>
+        </is>
+      </c>
+      <c r="D1943" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1943" t="inlineStr"/>
+      <c r="F1943" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g26</t>
+        </is>
+      </c>
+    </row>
+    <row r="1944">
+      <c r="A1944" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1944" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1944" t="inlineStr">
+        <is>
+          <t>FindingParts min</t>
+        </is>
+      </c>
+      <c r="D1944" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1944" t="inlineStr"/>
+      <c r="F1944" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g27</t>
+        </is>
+      </c>
+    </row>
+    <row r="1945">
+      <c r="A1945" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1945" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1945" t="inlineStr">
+        <is>
+          <t>PickingParts min</t>
+        </is>
+      </c>
+      <c r="D1945" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1945" t="inlineStr"/>
+      <c r="F1945" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g28</t>
+        </is>
+      </c>
+    </row>
+    <row r="1946">
+      <c r="A1946" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1946" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1946" t="inlineStr">
+        <is>
+          <t>PlacingParts min</t>
+        </is>
+      </c>
+      <c r="D1946" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1946" t="inlineStr"/>
+      <c r="F1946" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g29</t>
+        </is>
+      </c>
+    </row>
+    <row r="1947">
+      <c r="A1947" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1947" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1947" t="inlineStr">
+        <is>
+          <t>CountPickedReject14in</t>
+        </is>
+      </c>
+      <c r="D1947" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1947" t="inlineStr"/>
+      <c r="F1947" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1948">
+      <c r="A1948" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1948" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1948" t="inlineStr">
+        <is>
+          <t>temp_dsi</t>
+        </is>
+      </c>
+      <c r="D1948" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1948" t="inlineStr"/>
+      <c r="F1948" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g31</t>
+        </is>
+      </c>
+    </row>
+    <row r="1949">
+      <c r="A1949" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1949" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1949" t="inlineStr">
+        <is>
+          <t>temp_J1motor</t>
+        </is>
+      </c>
+      <c r="D1949" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1949" t="inlineStr"/>
+      <c r="F1949" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g32</t>
+        </is>
+      </c>
+    </row>
+    <row r="1950">
+      <c r="A1950" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1950" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1950" t="inlineStr">
+        <is>
+          <t>temp_J4motor</t>
+        </is>
+      </c>
+      <c r="D1950" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1950" t="inlineStr"/>
+      <c r="F1950" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g35</t>
+        </is>
+      </c>
+    </row>
+    <row r="1951">
+      <c r="A1951" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1951" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1951" t="inlineStr">
+        <is>
+          <t>temp_J6motor</t>
+        </is>
+      </c>
+      <c r="D1951" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1951" t="inlineStr"/>
+      <c r="F1951" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g37</t>
+        </is>
+      </c>
+    </row>
+    <row r="1952">
+      <c r="A1952" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1952" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1952" t="inlineStr">
+        <is>
+          <t>CountPickedRejectOTM</t>
+        </is>
+      </c>
+      <c r="D1952" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1952" t="inlineStr"/>
+      <c r="F1952" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g38</t>
+        </is>
+      </c>
+    </row>
+    <row r="1953">
+      <c r="A1953" t="inlineStr">
+        <is>
+          <t>2026-08-17T18:05:13</t>
+        </is>
+      </c>
+      <c r="B1953" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1953" t="inlineStr">
+        <is>
+          <t>CountPickedRejectPandral</t>
+        </is>
+      </c>
+      <c r="D1953" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1953" t="inlineStr"/>
+      <c r="F1953" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g39</t>
         </is>
       </c>
     </row>

</xml_diff>